<commit_message>
Introduction du TU MV C06
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS C06/CAS C06.xlsx
+++ b/VALIDATION/CAS C06/CAS C06.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS C06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358C68DD-FBB6-44FD-8078-7F297D778858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BBAFA2-31D7-49E9-9C70-1D4E281A0015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Général" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="Ah">Général!$E$74</definedName>
     <definedName name="AireA">Général!$E$15</definedName>
     <definedName name="Av">Général!$E$19</definedName>
     <definedName name="b">Général!$E$11</definedName>
@@ -33,24 +34,26 @@
     <definedName name="Fsk">Général!$J$8</definedName>
     <definedName name="fusc">Général!$E$34</definedName>
     <definedName name="Fy">Général!$J$4</definedName>
-    <definedName name="g">Général!$J$28</definedName>
-    <definedName name="GammaC">Général!$J$16</definedName>
-    <definedName name="GammaG">Général!$J$20</definedName>
-    <definedName name="GammaM0">Général!$J$14</definedName>
-    <definedName name="GammaM1">Général!$J$15</definedName>
-    <definedName name="GammaQ">Général!$J$21</definedName>
-    <definedName name="GammaS">Général!$J$17</definedName>
-    <definedName name="GammaV">Général!$J$18</definedName>
+    <definedName name="g">Général!$J$30</definedName>
+    <definedName name="GammaC">Général!$J$18</definedName>
+    <definedName name="GammaG">Général!$J$22</definedName>
+    <definedName name="GammaM0">Général!$J$16</definedName>
+    <definedName name="GammaM1">Général!$J$17</definedName>
+    <definedName name="GammaQ">Général!$J$23</definedName>
+    <definedName name="GammaS">Général!$J$19</definedName>
+    <definedName name="GammaV">Général!$J$20</definedName>
     <definedName name="hsc">Général!$E$32</definedName>
     <definedName name="Ht">Général!$E$10</definedName>
     <definedName name="hw">Général!$E$17</definedName>
+    <definedName name="Iy">Général!$E$22</definedName>
     <definedName name="Le">Général!$O$8</definedName>
     <definedName name="LL">Général!$E$4</definedName>
-    <definedName name="mDalle">Général!$J$32</definedName>
+    <definedName name="mDalle">Général!$J$34</definedName>
     <definedName name="MEd">Général!$N$48</definedName>
     <definedName name="MplRd">Général!$O$27</definedName>
     <definedName name="MplRd0">Général!$O$26</definedName>
-    <definedName name="mPro">Général!$J$33</definedName>
+    <definedName name="mPro">Général!$J$35</definedName>
+    <definedName name="n">Général!$E$72</definedName>
     <definedName name="Na">Général!$O$15</definedName>
     <definedName name="Nc">Général!$O$14</definedName>
     <definedName name="Nf">Général!$O$16</definedName>
@@ -73,8 +76,8 @@
     <definedName name="RatiozH">Général!$O$23</definedName>
     <definedName name="Rconnex">Général!$O$33</definedName>
     <definedName name="RcumPRd">Général!$O$32</definedName>
-    <definedName name="RhoA">Général!$J$26</definedName>
-    <definedName name="RhoC">Général!$J$27</definedName>
+    <definedName name="RhoA">Général!$J$28</definedName>
+    <definedName name="RhoC">Général!$J$29</definedName>
     <definedName name="rr">Général!$E$14</definedName>
     <definedName name="sxsc">Général!$E$35</definedName>
     <definedName name="tc">Général!$E$27</definedName>
@@ -85,8 +88,10 @@
     <definedName name="VplRd">Général!$O$29</definedName>
     <definedName name="Wel">Général!$E$21</definedName>
     <definedName name="Wpl">Général!$E$20</definedName>
+    <definedName name="zANE_1">Général!$E$78</definedName>
     <definedName name="zANP">Général!$O$22</definedName>
     <definedName name="zn">Général!$O$21</definedName>
+    <definedName name="zp">Général!$E$75</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -109,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="120">
   <si>
     <t>Poutre</t>
   </si>
@@ -433,6 +438,42 @@
   </si>
   <si>
     <t>ELU</t>
+  </si>
+  <si>
+    <t>MplRd profilé</t>
+  </si>
+  <si>
+    <t>n0</t>
+  </si>
+  <si>
+    <t>Propriétés élastiques</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Ah</t>
+  </si>
+  <si>
+    <t>zp</t>
+  </si>
+  <si>
+    <t>Hypothèse hors dalle</t>
+  </si>
+  <si>
+    <t>zANE</t>
+  </si>
+  <si>
+    <t>Hypothèse validée ?</t>
+  </si>
+  <si>
+    <t>Ih</t>
+  </si>
+  <si>
+    <t>Iy</t>
+  </si>
+  <si>
+    <t>cm4</t>
   </si>
 </sst>
 </file>
@@ -468,7 +509,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,6 +570,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE06520"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -557,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -619,12 +672,25 @@
     <xf numFmtId="166" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFE06520"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -953,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA8D444-109B-41E4-8631-33F090AACEB2}">
-  <dimension ref="C2:U61"/>
+  <dimension ref="C2:U96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="3:21" x14ac:dyDescent="0.25">
@@ -1153,6 +1219,13 @@
       <c r="F11" t="s">
         <v>6</v>
       </c>
+      <c r="I11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J11" s="26">
+        <f>210/Ecm</f>
+        <v>6.6717909812633494</v>
+      </c>
     </row>
     <row r="12" spans="3:21" x14ac:dyDescent="0.25">
       <c r="D12" s="2" t="s">
@@ -1164,12 +1237,6 @@
       <c r="F12" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
       <c r="M12" s="16"/>
       <c r="N12" s="16" t="s">
         <v>52</v>
@@ -1204,12 +1271,12 @@
       <c r="F14" t="s">
         <v>6</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J14" s="3">
-        <v>1</v>
-      </c>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
       <c r="N14" s="2" t="s">
         <v>53</v>
       </c>
@@ -1238,12 +1305,6 @@
       </c>
       <c r="F15" t="s">
         <v>12</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J15" s="3">
-        <v>1</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>55</v>
@@ -1272,10 +1333,10 @@
         <v>13</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J16" s="3">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>58</v>
@@ -1300,10 +1361,10 @@
         <v>6</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J17" s="3">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="3:16" x14ac:dyDescent="0.25">
@@ -1318,10 +1379,10 @@
         <v>6</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J18" s="3">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="N18" s="12" t="s">
         <v>59</v>
@@ -1342,7 +1403,12 @@
       <c r="F19" t="s">
         <v>12</v>
       </c>
-      <c r="I19" s="2"/>
+      <c r="I19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J19" s="3">
+        <v>1.1499999999999999</v>
+      </c>
     </row>
     <row r="20" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D20" s="2" t="s">
@@ -1355,10 +1421,10 @@
         <v>18</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J20" s="3">
-        <v>1.35</v>
+        <v>1.25</v>
       </c>
       <c r="N20" s="12" t="s">
         <v>62</v>
@@ -1378,12 +1444,7 @@
       <c r="F21" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="J21" s="3">
-        <v>1.5</v>
-      </c>
+      <c r="I21" s="2"/>
       <c r="N21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1396,7 +1457,21 @@
       </c>
     </row>
     <row r="22" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="I22" s="2"/>
+      <c r="D22" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="3">
+        <v>48200</v>
+      </c>
+      <c r="F22" t="s">
+        <v>119</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J22" s="3">
+        <v>1.35</v>
+      </c>
       <c r="N22" s="12" t="s">
         <v>64</v>
       </c>
@@ -1409,7 +1484,12 @@
       </c>
     </row>
     <row r="23" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="I23" s="2"/>
+      <c r="I23" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J23" s="3">
+        <v>1.5</v>
+      </c>
       <c r="N23" s="12" t="s">
         <v>65</v>
       </c>
@@ -1425,12 +1505,7 @@
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
+      <c r="I24" s="2"/>
       <c r="N24" s="12" t="s">
         <v>66</v>
       </c>
@@ -1452,15 +1527,12 @@
       <c r="F26" t="s">
         <v>6</v>
       </c>
-      <c r="I26" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J26" s="3">
-        <v>7850</v>
-      </c>
-      <c r="K26" t="s">
-        <v>42</v>
-      </c>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
       <c r="N26" s="12" t="s">
         <v>67</v>
       </c>
@@ -1483,15 +1555,7 @@
       <c r="F27" t="s">
         <v>6</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="J27" s="3">
-        <v>2500</v>
-      </c>
-      <c r="K27" t="s">
-        <v>42</v>
-      </c>
+      <c r="I27" s="2"/>
       <c r="N27" s="12" t="s">
         <v>68</v>
       </c>
@@ -1505,16 +1569,25 @@
     </row>
     <row r="28" spans="3:16" x14ac:dyDescent="0.25">
       <c r="I28" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J28" s="3">
-        <v>9.81</v>
+        <v>7850</v>
       </c>
       <c r="K28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="I29" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J29" s="3">
+        <v>2500</v>
+      </c>
+      <c r="K29" t="s">
+        <v>42</v>
+      </c>
       <c r="N29" s="12" t="s">
         <v>70</v>
       </c>
@@ -1533,10 +1606,14 @@
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="I31" s="12" t="s">
-        <v>86</v>
+      <c r="I30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J30" s="3">
+        <v>9.81</v>
+      </c>
+      <c r="K30" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="3:16" x14ac:dyDescent="0.25">
@@ -1549,16 +1626,6 @@
       <c r="F32" t="s">
         <v>6</v>
       </c>
-      <c r="I32" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="J32" s="15">
-        <f>d*td*LL*RhoC/1000</f>
-        <v>8925</v>
-      </c>
-      <c r="K32" t="s">
-        <v>87</v>
-      </c>
       <c r="N32" s="2" t="s">
         <v>100</v>
       </c>
@@ -1581,14 +1648,7 @@
         <v>6</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="J33" s="20">
-        <f>AireA/1000^2*LL*RhoA</f>
-        <v>1269.5821246103822</v>
-      </c>
-      <c r="K33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>101</v>
@@ -1611,6 +1671,16 @@
       <c r="F34" t="s">
         <v>24</v>
       </c>
+      <c r="I34" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="J34" s="15">
+        <f>d*td*LL*RhoC/1000</f>
+        <v>8925</v>
+      </c>
+      <c r="K34" t="s">
+        <v>87</v>
+      </c>
       <c r="N34" s="2" t="s">
         <v>102</v>
       </c>
@@ -1633,6 +1703,16 @@
         <f>6*td</f>
         <v>900</v>
       </c>
+      <c r="I35" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="J35" s="20">
+        <f>AireA/1000^2*LL*RhoA</f>
+        <v>1269.5821246103822</v>
+      </c>
+      <c r="K35" t="s">
+        <v>87</v>
+      </c>
       <c r="O35" s="13"/>
     </row>
     <row r="36" spans="3:16" x14ac:dyDescent="0.25">
@@ -1655,7 +1735,16 @@
       <c r="O37" s="13"/>
     </row>
     <row r="38" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="O38" s="13"/>
+      <c r="N38" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="O38" s="25">
+        <f>Wpl*Fy/GammaM0/1000</f>
+        <v>1009.24</v>
+      </c>
+      <c r="P38" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="39" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D39" s="12" t="s">
@@ -1909,6 +1998,156 @@
         <v>242.43597418363882</v>
       </c>
     </row>
+    <row r="70" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C70" s="27"/>
+      <c r="D70" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="E70" s="27"/>
+      <c r="F70" s="27"/>
+    </row>
+    <row r="72" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D72" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E72" s="3">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="74" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D74" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E74" s="20">
+        <f>AireA+beff*td*1000/n</f>
+        <v>21552.157639766898</v>
+      </c>
+      <c r="F74" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="75" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D75" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E75" s="15">
+        <f>Ht/2+td</f>
+        <v>400</v>
+      </c>
+      <c r="F75" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D76" s="2"/>
+      <c r="E76" s="13"/>
+    </row>
+    <row r="77" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D77" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E77" s="13"/>
+    </row>
+    <row r="78" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D78" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E78" s="18">
+        <f>zp*AireA/Ah+beff*td^2*1000/2/n/Ah</f>
+        <v>249.20303320335444</v>
+      </c>
+      <c r="F78" t="s">
+        <v>6</v>
+      </c>
+      <c r="G78" s="17">
+        <f>zANE_1-td</f>
+        <v>99.203033203354437</v>
+      </c>
+    </row>
+    <row r="79" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D79" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E79" s="15" t="str">
+        <f>IF(zANE_1&gt;td,Oui,Non)</f>
+        <v>oui</v>
+      </c>
+    </row>
+    <row r="80" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D80" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E80" s="20">
+        <f>Iy+AireA/100*(zp-zANE_1)^2/10^2+beff*100*td/10/3/n*((td/10)^2+3*zANE_1/100*(zANE_1-td))</f>
+        <v>106690.98579109021</v>
+      </c>
+      <c r="F80" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="81" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D81" s="2"/>
+      <c r="E81" s="13"/>
+    </row>
+    <row r="82" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D82" s="2"/>
+      <c r="E82" s="13"/>
+    </row>
+    <row r="83" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D83" s="2"/>
+      <c r="E83" s="13"/>
+    </row>
+    <row r="84" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D84" s="2"/>
+      <c r="E84" s="13"/>
+    </row>
+    <row r="85" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D85" s="2"/>
+      <c r="E85" s="13"/>
+    </row>
+    <row r="86" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D86" s="2"/>
+      <c r="E86" s="13"/>
+    </row>
+    <row r="87" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D87" s="2"/>
+      <c r="E87" s="13"/>
+    </row>
+    <row r="88" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D88" s="2"/>
+      <c r="E88" s="13"/>
+    </row>
+    <row r="89" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D89" s="2"/>
+      <c r="E89" s="13"/>
+    </row>
+    <row r="90" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D90" s="2"/>
+      <c r="E90" s="13"/>
+    </row>
+    <row r="91" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D91" s="2"/>
+      <c r="E91" s="13"/>
+    </row>
+    <row r="92" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D92" s="2"/>
+      <c r="E92" s="13"/>
+    </row>
+    <row r="93" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D93" s="2"/>
+      <c r="E93" s="13"/>
+    </row>
+    <row r="94" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D94" s="2"/>
+      <c r="E94" s="13"/>
+    </row>
+    <row r="95" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D95" s="2"/>
+      <c r="E95" s="13"/>
+    </row>
+    <row r="96" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E96" s="13"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>

<commit_message>
Avancement 02 01 25 - Calcul ferraillage Trans - Cofraplus 220
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS C06/CAS C06.xlsx
+++ b/VALIDATION/CAS C06/CAS C06.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS C06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BBAFA2-31D7-49E9-9C70-1D4E281A0015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFBE7A3-9F0E-4AC6-A0FE-4765BEE10A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
   </bookViews>
   <sheets>
     <sheet name="Général" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Ah">Général!$E$74</definedName>
+    <definedName name="Ah">Général!$E$76</definedName>
     <definedName name="AireA">Général!$E$15</definedName>
     <definedName name="Av">Général!$E$19</definedName>
     <definedName name="b">Général!$E$11</definedName>
+    <definedName name="b0">Général!$E$92</definedName>
     <definedName name="beff">Général!$O$4</definedName>
     <definedName name="bei">Général!$O$7</definedName>
     <definedName name="BetaExt">Général!$O$9</definedName>
@@ -46,6 +47,7 @@
     <definedName name="Ht">Général!$E$10</definedName>
     <definedName name="hw">Général!$E$17</definedName>
     <definedName name="Iy">Général!$E$22</definedName>
+    <definedName name="ksfaa">Général!$E$93</definedName>
     <definedName name="Le">Général!$O$8</definedName>
     <definedName name="LL">Général!$E$4</definedName>
     <definedName name="mDalle">Général!$J$34</definedName>
@@ -53,13 +55,14 @@
     <definedName name="MplRd">Général!$O$27</definedName>
     <definedName name="MplRd0">Général!$O$26</definedName>
     <definedName name="mPro">Général!$J$35</definedName>
-    <definedName name="n">Général!$E$72</definedName>
+    <definedName name="n">Général!$E$74</definedName>
     <definedName name="Na">Général!$O$15</definedName>
     <definedName name="Nc">Général!$O$14</definedName>
     <definedName name="Nf">Général!$O$16</definedName>
     <definedName name="Non">Général!$S$3</definedName>
     <definedName name="nr">Général!$E$36</definedName>
     <definedName name="Nu">Général!$J$5</definedName>
+    <definedName name="NuT">Général!$E$91</definedName>
     <definedName name="Oui">Général!$S$2</definedName>
     <definedName name="p">Général!$O$20</definedName>
     <definedName name="PRd">Général!$E$41</definedName>
@@ -88,10 +91,10 @@
     <definedName name="VplRd">Général!$O$29</definedName>
     <definedName name="Wel">Général!$E$21</definedName>
     <definedName name="Wpl">Général!$E$20</definedName>
-    <definedName name="zANE_1">Général!$E$78</definedName>
+    <definedName name="zANE_1">Général!$E$80</definedName>
     <definedName name="zANP">Général!$O$22</definedName>
     <definedName name="zn">Général!$O$21</definedName>
-    <definedName name="zp">Général!$E$75</definedName>
+    <definedName name="zp">Général!$E$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -114,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="144">
   <si>
     <t>Poutre</t>
   </si>
@@ -474,15 +477,88 @@
   </si>
   <si>
     <t>cm4</t>
+  </si>
+  <si>
+    <t>Flèches</t>
+  </si>
+  <si>
+    <t>Flèche (mm)</t>
+  </si>
+  <si>
+    <t>q (kN/m)</t>
+  </si>
+  <si>
+    <t>Iy (cm4)</t>
+  </si>
+  <si>
+    <t>h0</t>
+  </si>
+  <si>
+    <t>Armatures transversales</t>
+  </si>
+  <si>
+    <t>Flux global</t>
+  </si>
+  <si>
+    <t>Flux / côté</t>
+  </si>
+  <si>
+    <t>Aire</t>
+  </si>
+  <si>
+    <t>a-a</t>
+  </si>
+  <si>
+    <t>b-b</t>
+  </si>
+  <si>
+    <t>d (mm)</t>
+  </si>
+  <si>
+    <t>TEd (MPa)</t>
+  </si>
+  <si>
+    <t>Theta (°)</t>
+  </si>
+  <si>
+    <t>TRd (MPa)</t>
+  </si>
+  <si>
+    <t>At+Ab</t>
+  </si>
+  <si>
+    <t>2 Ab</t>
+  </si>
+  <si>
+    <t>Aire (cm2/m)</t>
+  </si>
+  <si>
+    <t>Ab mini</t>
+  </si>
+  <si>
+    <t>cm2/m</t>
+  </si>
+  <si>
+    <t>At mini</t>
+  </si>
+  <si>
+    <t>Critère béton</t>
+  </si>
+  <si>
+    <t>b0</t>
+  </si>
+  <si>
+    <t>ksf a-a</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -509,7 +585,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -582,6 +658,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -610,7 +698,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -637,9 +725,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -650,7 +735,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -669,17 +754,30 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1019,7 +1117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA8D444-109B-41E4-8631-33F090AACEB2}">
-  <dimension ref="C2:U96"/>
+  <dimension ref="C2:U106"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="3:21" x14ac:dyDescent="0.25">
@@ -1041,12 +1139,12 @@
       </c>
       <c r="O2" s="10"/>
       <c r="P2" s="10"/>
-      <c r="S2" s="15" t="s">
+      <c r="S2" s="14" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="3" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="S3" s="15" t="s">
+      <c r="S3" s="14" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1137,7 +1235,7 @@
       <c r="N7" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="O7" s="15">
+      <c r="O7" s="14">
         <f>MIN(Le/8,d/2)</f>
         <v>0.85</v>
       </c>
@@ -1158,7 +1256,7 @@
       <c r="N8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="O8" s="15">
+      <c r="O8" s="14">
         <f>LL</f>
         <v>14</v>
       </c>
@@ -1180,10 +1278,10 @@
       <c r="K9" t="s">
         <v>30</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="O9" s="17">
+      <c r="O9" s="16">
         <f>MIN(1,(0.55+0.025*Le/bei))</f>
         <v>0.96176470588235308</v>
       </c>
@@ -1222,7 +1320,7 @@
       <c r="I11" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="26">
+      <c r="J11" s="25">
         <f>210/Ecm</f>
         <v>6.6717909812633494</v>
       </c>
@@ -1237,18 +1335,18 @@
       <c r="F12" t="s">
         <v>6</v>
       </c>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16" t="s">
+      <c r="M12" s="15"/>
+      <c r="N12" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="O12" s="16"/>
-      <c r="P12" s="16"/>
-      <c r="R12" s="23"/>
-      <c r="S12" s="23" t="s">
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="R12" s="22"/>
+      <c r="S12" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="T12" s="23"/>
-      <c r="U12" s="23"/>
+      <c r="T12" s="22"/>
+      <c r="U12" s="22"/>
     </row>
     <row r="13" spans="3:21" x14ac:dyDescent="0.25">
       <c r="D13" s="2" t="s">
@@ -1290,7 +1388,7 @@
       <c r="S14" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="T14" s="24">
+      <c r="T14" s="23">
         <f>MEd/MplRd</f>
         <v>0.5653623558103682</v>
       </c>
@@ -1319,7 +1417,7 @@
       <c r="S15" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="T15" s="24">
+      <c r="T15" s="23">
         <f>VEd/VplRd</f>
         <v>0.15246306944556504</v>
       </c>
@@ -1384,7 +1482,7 @@
       <c r="J18" s="3">
         <v>1.5</v>
       </c>
-      <c r="N18" s="12" t="s">
+      <c r="N18" s="2" t="s">
         <v>59</v>
       </c>
       <c r="O18" s="3" t="str">
@@ -1426,10 +1524,10 @@
       <c r="J20" s="3">
         <v>1.25</v>
       </c>
-      <c r="N20" s="12" t="s">
+      <c r="N20" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="O20" s="17">
+      <c r="O20" s="16">
         <f>(Na-Nc)/2/Nf</f>
         <v>0.57795262034401307</v>
       </c>
@@ -1448,7 +1546,7 @@
       <c r="N21" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="O21" s="17">
+      <c r="O21" s="16">
         <f>p*tf</f>
         <v>9.2472419255042091</v>
       </c>
@@ -1472,10 +1570,10 @@
       <c r="J22" s="3">
         <v>1.35</v>
       </c>
-      <c r="N22" s="12" t="s">
+      <c r="N22" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="O22" s="20">
+      <c r="O22" s="19">
         <f>td+zn</f>
         <v>159.2472419255042</v>
       </c>
@@ -1490,10 +1588,10 @@
       <c r="J23" s="3">
         <v>1.5</v>
       </c>
-      <c r="N23" s="12" t="s">
+      <c r="N23" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="O23" s="17">
+      <c r="O23" s="16">
         <f>zANP/(Ht+td)</f>
         <v>0.244995756808468</v>
       </c>
@@ -1506,10 +1604,10 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="I24" s="2"/>
-      <c r="N24" s="12" t="s">
+      <c r="N24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="O24" s="17">
+      <c r="O24" s="16">
         <f>1-0.15*(RatiozH-0.15)/(0.4-0.15)</f>
         <v>0.94300254591491917</v>
       </c>
@@ -1533,10 +1631,10 @@
       </c>
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
-      <c r="N26" s="12" t="s">
+      <c r="N26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="O26" s="20">
+      <c r="O26" s="19">
         <f>(Nc*(tc/2+td-tc)+Na*Ht/2+(Nc-Na)*zn/2)/1000</f>
         <v>1591.5685721161435</v>
       </c>
@@ -1548,7 +1646,7 @@
       <c r="D27" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="14">
         <f>td</f>
         <v>150</v>
       </c>
@@ -1556,10 +1654,10 @@
         <v>6</v>
       </c>
       <c r="I27" s="2"/>
-      <c r="N27" s="12" t="s">
+      <c r="N27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="O27" s="20">
+      <c r="O27" s="19">
         <f>BetaMpl*MplRd0</f>
         <v>1500.853215503696</v>
       </c>
@@ -1588,10 +1686,10 @@
       <c r="K29" t="s">
         <v>42</v>
       </c>
-      <c r="N29" s="12" t="s">
+      <c r="N29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O29" s="20">
+      <c r="O29" s="19">
         <f>Av*Fy/SQRT(3)/GammaM0/1000</f>
         <v>1590.129170724832</v>
       </c>
@@ -1629,7 +1727,7 @@
       <c r="N32" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="O32" s="22">
+      <c r="O32" s="21">
         <f>nr*PRd*LL/2/(sxsc/1000)</f>
         <v>3984.29763465519</v>
       </c>
@@ -1647,13 +1745,13 @@
       <c r="F33" t="s">
         <v>6</v>
       </c>
-      <c r="I33" s="12" t="s">
+      <c r="I33" s="2" t="s">
         <v>86</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="O33" s="14">
+      <c r="O33" s="13">
         <f>MIN(Na,Nc)</f>
         <v>3612.4999999999995</v>
       </c>
@@ -1671,10 +1769,10 @@
       <c r="F34" t="s">
         <v>24</v>
       </c>
-      <c r="I34" s="12" t="s">
+      <c r="I34" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J34" s="15">
+      <c r="J34" s="14">
         <f>d*td*LL*RhoC/1000</f>
         <v>8925</v>
       </c>
@@ -1684,7 +1782,7 @@
       <c r="N34" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="O34" s="21">
+      <c r="O34" s="20">
         <f>RcumPRd/Rconnex</f>
         <v>1.1029197604581842</v>
       </c>
@@ -1699,21 +1797,21 @@
       <c r="F35" t="s">
         <v>6</v>
       </c>
-      <c r="G35" s="14">
+      <c r="G35" s="13">
         <f>6*td</f>
         <v>900</v>
       </c>
-      <c r="I35" s="12" t="s">
+      <c r="I35" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J35" s="20">
+      <c r="J35" s="19">
         <f>AireA/1000^2*LL*RhoA</f>
         <v>1269.5821246103822</v>
       </c>
       <c r="K35" t="s">
         <v>87</v>
       </c>
-      <c r="O35" s="13"/>
+      <c r="O35" s="12"/>
     </row>
     <row r="36" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D36" s="2" t="s">
@@ -1722,23 +1820,23 @@
       <c r="E36" s="3">
         <v>2</v>
       </c>
-      <c r="O36" s="13"/>
+      <c r="O36" s="12"/>
     </row>
     <row r="37" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D37" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E37" s="17">
+      <c r="E37" s="16">
         <f>hsc/dsc</f>
         <v>5.6818181818181817</v>
       </c>
-      <c r="O37" s="13"/>
+      <c r="O37" s="12"/>
     </row>
     <row r="38" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N38" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="O38" s="25">
+      <c r="O38" s="24">
         <f>Wpl*Fy/GammaM0/1000</f>
         <v>1009.24</v>
       </c>
@@ -1747,46 +1845,46 @@
       </c>
     </row>
     <row r="39" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="D39" s="12" t="s">
+      <c r="D39" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E39" s="19">
+      <c r="E39" s="18">
         <f>0.8*fusc*PI()*dsc^2/4000/GammaV</f>
         <v>109.47822079229711</v>
       </c>
       <c r="F39" t="s">
         <v>54</v>
       </c>
-      <c r="O39" s="13"/>
+      <c r="O39" s="12"/>
     </row>
     <row r="40" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="D40" s="12" t="s">
+      <c r="D40" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E40" s="19">
+      <c r="E40" s="18">
         <f>0.29*dsc^2*SQRT(Ecm*1000*Fck)/GammaV/1000</f>
         <v>99.607440866379747</v>
       </c>
       <c r="F40" t="s">
         <v>54</v>
       </c>
-      <c r="O40" s="13"/>
+      <c r="O40" s="12"/>
     </row>
     <row r="41" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="D41" s="12" t="s">
+      <c r="D41" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E41" s="19">
+      <c r="E41" s="18">
         <f>MIN(PRdc,PRds)</f>
         <v>99.607440866379747</v>
       </c>
       <c r="F41" t="s">
         <v>54</v>
       </c>
-      <c r="O41" s="13"/>
+      <c r="O41" s="12"/>
     </row>
     <row r="42" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="O42" s="13"/>
+      <c r="O42" s="12"/>
     </row>
     <row r="44" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C44" s="1"/>
@@ -1809,7 +1907,7 @@
       <c r="D46" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E46" s="17">
+      <c r="E46" s="16">
         <f>mDalle/LL*g/1000</f>
         <v>6.2538749999999999</v>
       </c>
@@ -1819,7 +1917,7 @@
       <c r="M46" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="N46" s="18">
+      <c r="N46" s="17">
         <f>GammaG*(q_G1+q_G2)+GammaQ*q_Q1</f>
         <v>34.633710597662684</v>
       </c>
@@ -1831,7 +1929,7 @@
       <c r="D47" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E47" s="17">
+      <c r="E47" s="16">
         <f>mPro/LL*g/1000</f>
         <v>0.88961433160198933</v>
       </c>
@@ -1843,7 +1941,7 @@
       <c r="D48" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E48" s="17">
+      <c r="E48" s="16">
         <f>q1Dalle+q1Pro</f>
         <v>7.1434893316019892</v>
       </c>
@@ -1853,7 +1951,7 @@
       <c r="M48" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="N48" s="19">
+      <c r="N48" s="18">
         <f>qULS*LL^2/8</f>
         <v>848.52590964273577</v>
       </c>
@@ -1865,10 +1963,10 @@
       <c r="C49" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D49" s="12" t="s">
+      <c r="D49" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E49" s="15">
+      <c r="E49" s="14">
         <f>Qs_G2*d</f>
         <v>3.4</v>
       </c>
@@ -1887,7 +1985,7 @@
       <c r="M49" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="N49" s="19">
+      <c r="N49" s="18">
         <f>qULS*LL/2</f>
         <v>242.43597418363879</v>
       </c>
@@ -1899,10 +1997,10 @@
       <c r="C50" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D50" s="12" t="s">
+      <c r="D50" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E50" s="15">
+      <c r="E50" s="14">
         <f>Qs_Q1*d</f>
         <v>13.6</v>
       </c>
@@ -1920,13 +2018,13 @@
       </c>
     </row>
     <row r="57" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="E57" s="14" t="s">
+      <c r="E57" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="F57" s="14" t="s">
+      <c r="F57" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="G57" s="14" t="s">
+      <c r="G57" s="13" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1934,15 +2032,15 @@
       <c r="D58" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E58" s="21">
+      <c r="E58" s="20">
         <f>q_G1</f>
         <v>7.1434893316019892</v>
       </c>
-      <c r="F58" s="21">
+      <c r="F58" s="20">
         <f>E58*LL^2/8</f>
         <v>175.01548862424875</v>
       </c>
-      <c r="G58" s="21">
+      <c r="G58" s="20">
         <f>E58*LL/2</f>
         <v>50.004425321213922</v>
       </c>
@@ -1951,15 +2049,15 @@
       <c r="D59" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E59" s="21">
+      <c r="E59" s="20">
         <f>q_G2</f>
         <v>3.4</v>
       </c>
-      <c r="F59" s="21">
+      <c r="F59" s="20">
         <f>E59*LL^2/8</f>
         <v>83.3</v>
       </c>
-      <c r="G59" s="21">
+      <c r="G59" s="20">
         <f>E59*LL/2</f>
         <v>23.8</v>
       </c>
@@ -1968,185 +2066,400 @@
       <c r="D60" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E60" s="21">
+      <c r="E60" s="20">
         <f>q_Q1</f>
         <v>13.6</v>
       </c>
-      <c r="F60" s="21">
+      <c r="F60" s="20">
         <f>E60*LL^2/8</f>
         <v>333.2</v>
       </c>
-      <c r="G60" s="21">
+      <c r="G60" s="20">
         <f>E60*LL/2</f>
         <v>95.2</v>
       </c>
     </row>
     <row r="61" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="D61" s="12" t="s">
+      <c r="D61" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E61" s="21">
+      <c r="E61" s="20">
         <f>GammaG*(E58+E59)+GammaQ*E60</f>
         <v>34.633710597662684</v>
       </c>
-      <c r="F61" s="21">
+      <c r="F61" s="20">
         <f>GammaG*(F58+F59)+GammaQ*F60</f>
         <v>848.52590964273577</v>
       </c>
-      <c r="G61" s="21">
+      <c r="G61" s="20">
         <f>GammaG*(G58+G59)+GammaQ*G60</f>
         <v>242.43597418363882</v>
       </c>
     </row>
-    <row r="70" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C70" s="27"/>
-      <c r="D70" s="28" t="s">
+    <row r="70" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C70" s="26"/>
+      <c r="D70" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="E70" s="27"/>
-      <c r="F70" s="27"/>
-    </row>
-    <row r="72" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="E70" s="26"/>
+      <c r="F70" s="26"/>
+      <c r="L70" s="28"/>
+      <c r="M70" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="N70" s="28"/>
+      <c r="O70" s="28"/>
+    </row>
+    <row r="72" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D72" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E72" s="14">
+        <f>2*beff*1000*td/(2*beff*1000-b)</f>
+        <v>159.375</v>
+      </c>
+      <c r="F72" t="s">
+        <v>6</v>
+      </c>
+      <c r="M72" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="N72" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="O72" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="73" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="L73" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="M73" s="13">
+        <v>105214</v>
+      </c>
+      <c r="N73" s="13">
+        <f>M73</f>
+        <v>105214</v>
+      </c>
+      <c r="O73" s="13">
+        <v>148643</v>
+      </c>
+    </row>
+    <row r="74" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="D74" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E72" s="3">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row r="74" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D74" s="2" t="s">
+      <c r="E74" s="3">
+        <v>26.7</v>
+      </c>
+      <c r="L74" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="M74" s="20">
+        <f>E58</f>
+        <v>7.1434893316019892</v>
+      </c>
+      <c r="N74" s="20">
+        <f>E59</f>
+        <v>3.4</v>
+      </c>
+      <c r="O74" s="20">
+        <f>E60</f>
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="75" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="L75" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="M75" s="20">
+        <f>5/384*M74*LL^4/(Ey*M73/100)*1000^2</f>
+        <v>16.172177397834428</v>
+      </c>
+      <c r="N75" s="20">
+        <f>5/384*N74*LL^4/(Ey*N73/100)*1000^2</f>
+        <v>7.697275183066048</v>
+      </c>
+      <c r="O75" s="20">
+        <f>5/384*O74*LL^4/(Ey*O73/100)*1000^2</f>
+        <v>21.79345441389399</v>
+      </c>
+    </row>
+    <row r="76" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="D76" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E74" s="20">
+      <c r="E76" s="19">
         <f>AireA+beff*td*1000/n</f>
-        <v>21552.157639766898</v>
-      </c>
-      <c r="F74" t="s">
+        <v>21102.719437519707</v>
+      </c>
+      <c r="F76" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D75" s="2" t="s">
+    <row r="77" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="D77" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E75" s="15">
+      <c r="E77" s="14">
         <f>Ht/2+td</f>
         <v>400</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F77" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D76" s="2"/>
-      <c r="E76" s="13"/>
-    </row>
-    <row r="77" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D77" s="2" t="s">
+    <row r="78" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="D78" s="2"/>
+      <c r="E78" s="12"/>
+    </row>
+    <row r="79" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="D79" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E77" s="13"/>
-    </row>
-    <row r="78" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D78" s="2" t="s">
+      <c r="E79" s="12"/>
+    </row>
+    <row r="80" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="D80" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E78" s="18">
+      <c r="E80" s="17">
         <f>zp*AireA/Ah+beff*td^2*1000/2/n/Ah</f>
-        <v>249.20303320335444</v>
-      </c>
-      <c r="F78" t="s">
+        <v>252.91314735715974</v>
+      </c>
+      <c r="F80" t="s">
         <v>6</v>
       </c>
-      <c r="G78" s="17">
+      <c r="G80" s="16">
         <f>zANE_1-td</f>
-        <v>99.203033203354437</v>
-      </c>
-    </row>
-    <row r="79" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D79" s="2" t="s">
+        <v>102.91314735715974</v>
+      </c>
+    </row>
+    <row r="81" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D81" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E79" s="15" t="str">
+      <c r="E81" s="14" t="str">
         <f>IF(zANE_1&gt;td,Oui,Non)</f>
         <v>oui</v>
       </c>
     </row>
-    <row r="80" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D80" s="2" t="s">
+    <row r="82" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D82" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E80" s="20">
+      <c r="E82" s="19">
         <f>Iy+AireA/100*(zp-zANE_1)^2/10^2+beff*100*td/10/3/n*((td/10)^2+3*zANE_1/100*(zANE_1-td))</f>
-        <v>106690.98579109021</v>
-      </c>
-      <c r="F80" t="s">
+        <v>105213.77186226446</v>
+      </c>
+      <c r="F82" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="81" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D81" s="2"/>
-      <c r="E81" s="13"/>
-    </row>
-    <row r="82" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D82" s="2"/>
-      <c r="E82" s="13"/>
-    </row>
-    <row r="83" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D83" s="2"/>
-      <c r="E83" s="13"/>
-    </row>
-    <row r="84" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E83" s="12"/>
+    </row>
+    <row r="84" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D84" s="2"/>
-      <c r="E84" s="13"/>
-    </row>
-    <row r="85" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E84" s="12"/>
+    </row>
+    <row r="85" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D85" s="2"/>
-      <c r="E85" s="13"/>
-    </row>
-    <row r="86" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E85" s="12"/>
+    </row>
+    <row r="86" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D86" s="2"/>
-      <c r="E86" s="13"/>
-    </row>
-    <row r="87" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D87" s="2"/>
-      <c r="E87" s="13"/>
-    </row>
-    <row r="88" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E86" s="12"/>
+    </row>
+    <row r="87" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C87" s="30"/>
+      <c r="D87" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="E87" s="30"/>
+      <c r="F87" s="30"/>
+    </row>
+    <row r="88" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D88" s="2"/>
-      <c r="E88" s="13"/>
-    </row>
-    <row r="89" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D89" s="2"/>
-      <c r="E89" s="13"/>
-    </row>
-    <row r="90" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D90" s="2"/>
-      <c r="E90" s="13"/>
-    </row>
-    <row r="91" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D91" s="2"/>
-      <c r="E91" s="13"/>
-    </row>
-    <row r="92" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D92" s="2"/>
-      <c r="E92" s="13"/>
-    </row>
-    <row r="93" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D93" s="2"/>
-      <c r="E93" s="13"/>
-    </row>
-    <row r="94" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D94" s="2"/>
-      <c r="E94" s="13"/>
-    </row>
-    <row r="95" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D95" s="2"/>
-      <c r="E95" s="13"/>
-    </row>
-    <row r="96" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E96" s="13"/>
+      <c r="E88" s="12"/>
+    </row>
+    <row r="89" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D89" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E89" s="18">
+        <f>nr*PRd/(sxsc/1000)</f>
+        <v>569.18537637931286</v>
+      </c>
+      <c r="F89" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D90" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E90" s="18">
+        <f>E89/2</f>
+        <v>284.59268818965643</v>
+      </c>
+      <c r="F90" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D91" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E91" s="14">
+        <f>0.6*(1-Fck/250)</f>
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="92" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D92" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="E92" s="14">
+        <f>2.5*dsc</f>
+        <v>55</v>
+      </c>
+      <c r="F92" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="93" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D93" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="E93" s="34">
+        <f>(beff*1000-b0)/2/(beff*1000)</f>
+        <v>0.48382352941176471</v>
+      </c>
+    </row>
+    <row r="96" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D96" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E96" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F96" s="13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="97" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D97" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E97" s="13">
+        <f>tc</f>
+        <v>150</v>
+      </c>
+      <c r="F97" s="13">
+        <f>2*hsc+2.5*dsc+dsc</f>
+        <v>327</v>
+      </c>
+    </row>
+    <row r="98" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D98" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E98" s="32">
+        <f>E89/E97*ksfaa</f>
+        <v>1.8359018512626857</v>
+      </c>
+      <c r="F98" s="32">
+        <f>E89/F97</f>
+        <v>1.7406280623220576</v>
+      </c>
+    </row>
+    <row r="99" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D99" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E99" s="32">
+        <v>27</v>
+      </c>
+      <c r="F99" s="32">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="100" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D100" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E100" s="32">
+        <f>NuT*Fck/GammaC*SIN(E99*PI()/180)*COS(E99*PI()/180)</f>
+        <v>3.6405764746872631</v>
+      </c>
+      <c r="F100" s="32">
+        <f>NuT*Fck/GammaC*SIN(F99*PI()/180)*COS(F99*PI()/180)</f>
+        <v>3.6405764746872631</v>
+      </c>
+    </row>
+    <row r="101" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D101" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E101" s="32">
+        <f>E98/E100</f>
+        <v>0.50428877515075288</v>
+      </c>
+      <c r="F101" s="32">
+        <f>F98/F100</f>
+        <v>0.47811880190528971</v>
+      </c>
+    </row>
+    <row r="102" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D102" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E102" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="F102" s="13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="103" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D103" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E103" s="20">
+        <f>E98*E97*TAN(E99*PI()/180)/(Fsk/GammaS)*10</f>
+        <v>3.2272635701733448</v>
+      </c>
+      <c r="F103" s="20">
+        <f>F98*F97*TAN(F99*PI()/180)/(Fsk/GammaS)*10</f>
+        <v>6.6703319991424745</v>
+      </c>
+    </row>
+    <row r="105" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D105" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E105" s="20">
+        <f>F103/2</f>
+        <v>3.3351659995712373</v>
+      </c>
+      <c r="F105" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="106" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D106" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E106" s="20">
+        <f>E103-E105</f>
+        <v>-0.10790242939789252</v>
+      </c>
+      <c r="F106" t="s">
+        <v>139</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Preparation du cas SFS02
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS C06/CAS C06.xlsx
+++ b/VALIDATION/CAS C06/CAS C06.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS C06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFBE7A3-9F0E-4AC6-A0FE-4765BEE10A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA11715-88F2-4F7C-8C0F-30F740904956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{A3CDA6BD-B8DC-4D29-AE10-FB35D2143514}"/>
   </bookViews>
   <sheets>
     <sheet name="Général" sheetId="1" r:id="rId1"/>
@@ -68,6 +68,7 @@
     <definedName name="PRd">Général!$E$41</definedName>
     <definedName name="PRdc">Général!$E$40</definedName>
     <definedName name="PRds">Général!$E$39</definedName>
+    <definedName name="Psi2Q">Général!$Q$71</definedName>
     <definedName name="q_G1">Général!$E$48</definedName>
     <definedName name="q_G2">Général!$E$49</definedName>
     <definedName name="q_Q1">Général!$E$50</definedName>
@@ -117,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="148">
   <si>
     <t>Poutre</t>
   </si>
@@ -549,6 +550,18 @@
   </si>
   <si>
     <t>ksf a-a</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>Psi 2</t>
+  </si>
+  <si>
+    <t>Global</t>
   </si>
 </sst>
 </file>
@@ -558,7 +571,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -698,7 +711,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -772,10 +785,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2096,7 +2106,7 @@
         <v>242.43597418363882</v>
       </c>
     </row>
-    <row r="70" spans="3:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C70" s="26"/>
       <c r="D70" s="27" t="s">
         <v>110</v>
@@ -2109,8 +2119,18 @@
       </c>
       <c r="N70" s="28"/>
       <c r="O70" s="28"/>
-    </row>
-    <row r="72" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="P70" s="28"/>
+      <c r="Q70" s="28"/>
+    </row>
+    <row r="71" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="P71" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q71" s="3">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="72" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D72" s="2" t="s">
         <v>124</v>
       </c>
@@ -2121,32 +2141,34 @@
       <c r="F72" t="s">
         <v>6</v>
       </c>
-      <c r="M72" s="14" t="s">
+      <c r="O72" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="P72" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q72" s="12" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="73" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="M73" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="N72" s="14" t="s">
+      <c r="N73" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="O72" s="14" t="s">
+      <c r="O73" s="14" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="73" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="L73" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="M73" s="13">
-        <v>105214</v>
-      </c>
-      <c r="N73" s="13">
-        <f>M73</f>
-        <v>105214</v>
-      </c>
-      <c r="O73" s="13">
-        <v>148643</v>
-      </c>
-    </row>
-    <row r="74" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="P73" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q73" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="74" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D74" s="2" t="s">
         <v>111</v>
       </c>
@@ -2154,39 +2176,47 @@
         <v>26.7</v>
       </c>
       <c r="L74" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="M74" s="13">
+        <v>105214</v>
+      </c>
+      <c r="N74" s="13">
+        <f>M74</f>
+        <v>105214</v>
+      </c>
+      <c r="O74" s="13">
+        <v>148643</v>
+      </c>
+      <c r="P74" s="13">
+        <f>N74</f>
+        <v>105214</v>
+      </c>
+      <c r="Q74" s="13"/>
+    </row>
+    <row r="75" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="L75" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="M74" s="20">
+      <c r="M75" s="20">
         <f>E58</f>
         <v>7.1434893316019892</v>
       </c>
-      <c r="N74" s="20">
+      <c r="N75" s="20">
         <f>E59</f>
         <v>3.4</v>
       </c>
-      <c r="O74" s="20">
+      <c r="O75" s="20">
         <f>E60</f>
         <v>13.6</v>
       </c>
-    </row>
-    <row r="75" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="L75" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="M75" s="20">
-        <f>5/384*M74*LL^4/(Ey*M73/100)*1000^2</f>
-        <v>16.172177397834428</v>
-      </c>
-      <c r="N75" s="20">
-        <f>5/384*N74*LL^4/(Ey*N73/100)*1000^2</f>
-        <v>7.697275183066048</v>
-      </c>
-      <c r="O75" s="20">
-        <f>5/384*O74*LL^4/(Ey*O73/100)*1000^2</f>
-        <v>21.79345441389399</v>
-      </c>
-    </row>
-    <row r="76" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="P75" s="20">
+        <f>O75</f>
+        <v>13.6</v>
+      </c>
+      <c r="Q75" s="13"/>
+    </row>
+    <row r="76" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D76" s="2" t="s">
         <v>112</v>
       </c>
@@ -2197,8 +2227,31 @@
       <c r="F76" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="77" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="L76" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="M76" s="20">
+        <f>5/384*M75*LL^4/(Ey*M74/100)*1000^2</f>
+        <v>16.172177397834428</v>
+      </c>
+      <c r="N76" s="20">
+        <f>5/384*N75*LL^4/(Ey*N74/100)*1000^2</f>
+        <v>7.697275183066048</v>
+      </c>
+      <c r="O76" s="20">
+        <f>5/384*O75*LL^4/(Ey*O74/100)*1000^2</f>
+        <v>21.79345441389399</v>
+      </c>
+      <c r="P76" s="20">
+        <f>5/384*P75*LL^4/(Ey*P74/100)*1000^2</f>
+        <v>30.789100732264192</v>
+      </c>
+      <c r="Q76" s="20">
+        <f>(1-Psi2Q)*O76+Psi2Q*P76</f>
+        <v>25.391712941242069</v>
+      </c>
+    </row>
+    <row r="77" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D77" s="2" t="s">
         <v>113</v>
       </c>
@@ -2210,17 +2263,17 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="3:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D78" s="2"/>
       <c r="E78" s="12"/>
     </row>
-    <row r="79" spans="3:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D79" s="2" t="s">
         <v>114</v>
       </c>
       <c r="E79" s="12"/>
     </row>
-    <row r="80" spans="3:15" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D80" s="2" t="s">
         <v>115</v>
       </c>
@@ -2319,7 +2372,7 @@
       </c>
     </row>
     <row r="92" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D92" s="33" t="s">
+      <c r="D92" s="2" t="s">
         <v>142</v>
       </c>
       <c r="E92" s="14">
@@ -2331,10 +2384,10 @@
       </c>
     </row>
     <row r="93" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D93" s="33" t="s">
+      <c r="D93" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E93" s="34">
+      <c r="E93" s="33">
         <f>(beff*1000-b0)/2/(beff*1000)</f>
         <v>0.48382352941176471</v>
       </c>

</xml_diff>